<commit_message>
feat(materiais): planilha modelo integrado de 5 anos com mapa das ligações
A planilha gratuita agora mostra as 8 ligações entre DRE, Balanço e Fluxo de
Caixa, conferidas ao vivo, além de Lucro x Caixa com gráfico, 5 exercícios
guiados e uma aba com a oferta e os links do curso Fundamentos.
Mesmo endereço do arquivo, então o link do e-mail do Brevo continua valendo.
A página de captura passa a descrever o conteúdo novo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/materiais/modelo-integrado-simplificado.xlsx
+++ b/public/materiais/modelo-integrado-simplificado.xlsx
@@ -12,7 +12,11 @@
     <sheet name="DRE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Balanço" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Fluxo de Caixa" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Checagem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ligações" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Checagem" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Lucro x Caixa" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Exercícios" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Curso Fundamentos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,10 +25,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="0 &quot;dias&quot;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,7 +45,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
@@ -48,7 +52,28 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00070D24"/>
-      <sz val="13"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001D4ED8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0015803D"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -58,8 +83,37 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00475569"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00070D24"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -85,39 +139,30 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00070D24"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001D4ED8"/>
+      <color rgb="00B45309"/>
       <sz val="11"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="0015803D"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
+      <color rgb="00070D24"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -139,8 +184,13 @@
         <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F59E0B"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -150,16 +200,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9DEE7"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9DEE7"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9DEE7"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D9DEE7"/>
       </bottom>
     </border>
     <border>
@@ -167,41 +217,103 @@
         <color rgb="00070D24"/>
       </top>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9DEE7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -216,6 +328,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00DCFCE7"/>
+          <bgColor rgb="00DCFCE7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -227,6 +340,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FEE2E2"/>
+          <bgColor rgb="00FEE2E2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -301,6 +415,151 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Lucro líquido x Caixa das operações (R$ mil)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Lucro x Caixa'!B6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="070D24"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="070D24"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Lucro x Caixa'!$D$5:$H$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Lucro x Caixa'!$D$6:$H$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Lucro x Caixa'!B10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="F59E0B"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="F59E0B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Lucro x Caixa'!$D$5:$H$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Lucro x Caixa'!$D$10:$H$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -593,201 +852,630 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C26"/>
+  <dimension ref="B2:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Modelo integrado simplificado: DRE, Balanço e Fluxo de Caixa</t>
+          <t>Modelo integrado: DRE, Balanço e Fluxo de Caixa conectados</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mude as premissas e veja os três demonstrativos se moverem juntos. Se o Balanço não fechar, a aba Checagem avisa.</t>
+          <t>Saber montar cada demonstrativo separado é a parte fácil. Aqui você vê as 8 ligações que fazem os três virarem um modelo só, e fecharem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Como usar</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Como usar</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Vá na aba Premissas e mude só as células azuis (receita, crescimento, custos, prazos...).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Vá na aba Premissas e mude só as células azuis (receita, crescimento, custos, prazos...).</t>
+          <t>Acompanhe a DRE, o Balanço e o Fluxo de Caixa. Nenhuma outra célula precisa ser digitada.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Acompanhe a DRE, o Balanço e o Fluxo de Caixa. Nenhuma outra célula precisa ser digitada.</t>
+          <t>Abra a aba Ligações: ela mostra de onde sai e onde chega cada número que conecta os demonstrativos.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Confira a aba Checagem: a diferença do Balanço tem que ser zero em todos os anos.</t>
+          <t>Faça os 5 experimentos da aba Exercícios e confira na aba Checagem que o modelo continua fechando.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cores das células</t>
+          <t>As abas</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Premissas: Os únicos números digitados do modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>DRE, Balanço, Fluxo de Caixa: Os três demonstrativos de 5 anos, ligados por fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Ligações: As 8 conexões entre os demonstrativos, conferidas ao vivo, com o porquê de cada uma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Checagem: Ativo = Passivo + PL, caixa e lucro conferidos em todos os anos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Lucro x Caixa: A ponte entre lucro e caixa, com gráfico e indicadores de prazo e margem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Exercícios: Cinco testes guiados, inclusive quebrar uma ligação de propósito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Cores das células</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>■</t>
         </is>
       </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Azul: premissa. É o único lugar onde você digita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>■</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Preto: fórmula calculada na própria aba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>■</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Verde: número que vem de outra aba. É aqui que os demonstrativos se conectam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>O que este modelo deixa de fora, de propósito</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Dívida e juros (e o efeito deles no caixa e no lucro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Dividendos e distribuição de lucro</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Estoques e o ciclo de caixa completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Cenários e análise de sensibilidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>No curso Fundamentos da Modelagem Financeira você monta o modelo do zero e adiciona cada uma dessas peças sem quebrar as ligações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Conheça o curso Fundamentos da Modelagem Financeira →</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Ou veja o que o curso inclui na aba Curso Fundamentos →</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Valores em R$ mil. Empresa-exemplo de 5 anos, sem dívida, para focar na ligação entre os demonstrativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Modelagem Financeira na Prática · mfnapratica.com.br</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId1"/>
+    <hyperlink ref="C32" location="'Curso Fundamentos'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:C38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Curso Fundamentos da Modelagem Financeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Você viu as ligações funcionando nesta planilha. No curso, você monta esse modelo do zero, sabendo de onde vem cada número.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Para quem trava em ligar os três demonstrativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>O Balanço não fecha e você passa horas caçando a diferença entre ativo e passivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>A empresa lucrou no ano, faltou dinheiro no banco e você não consegue explicar o porquê.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Você começou um curso longo, parou na metade e continua sem ligar os demonstrativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>O que você monta, aula por aula</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>A lógica central do modelo. Você sai com o mapa de como as abas se ligam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Azul: premissa. É o único lugar onde você digita.</t>
+          <t>DRE: a estrutura do resultado. Você sai com a DRE montada no modelo.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>■</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Preto: fórmula calculada na própria aba.</t>
+          <t>Balanço: a fotografia. Você sai com o Balanço estruturado.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>■</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Verde: número que vem de outra aba. É aqui que os demonstrativos se conectam.</t>
+          <t>DFC: do lucro ao caixa. Você sai com o Fluxo de Caixa pelo método indireto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Capital de giro. Você sai com o capital de giro ligado ao caixa.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>O que este modelo deixa de fora, de propósito</t>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>As conexões que integram tudo. Você sai com os três demonstrativos conectados.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Dívida e juros (e o efeito deles no caixa e no lucro)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Dividendos e distribuição de lucro</t>
+          <t>Montagem e validação. Você sai com um modelo que fecha, com checagem automática.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Estoques e o ciclo de caixa completo</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>O que está incluído</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Cenários e análise de sensibilidade</t>
+          <t>Módulo das 3 demonstrações conectadas</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="4" t="inlineStr"/>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>No curso Fundamentos da Modelagem Financeira você adiciona cada uma dessas peças sem quebrar o modelo.</t>
+          <t>Módulos complementares com novas aulas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Template do modelo integrado em Excel</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Conheça o curso Fundamentos da Modelagem Financeira →</t>
+      <c r="B23" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Bônus: Template Pro (vendido por R$ 97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Bônus: Starter Kit Financeiro (vendido por R$ 67,90)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Valores em R$ mil. Empresa-exemplo, sem dívida, para focar na ligação entre os demonstrativos.</t>
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Bônus: Planilha de prompts de IA</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Modelagem Financeira na Prática · mfnapratica.com.br</t>
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Certificado de conclusão</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Acesso vitalício</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" s="44" t="inlineStr">
+        <is>
+          <t>12x de R$ 19,67 no cartão, ou R$ 197 à vista</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Garantia de 7 dias: se não for para você, peça o reembolso na Hotmart e receba 100% de volta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Pré-requisito: noção do que são DRE, Balanço e Fluxo de Caixa, e Excel básico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="C34" s="45" t="inlineStr">
+        <is>
+          <t>Ver a página do curso →</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>https://www.mfnapratica.com.br/fundamentos?utm_source=planilha-gratuita&amp;utm_medium=isca&amp;utm_campaign=modelo-integrado&amp;utm_content=aba-curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="C37" s="45" t="inlineStr">
+        <is>
+          <t>Comprar agora →</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>https://pay.hotmart.com/F106435738T?src=planilha-gratuita</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -806,7 +1494,7 @@
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -824,19 +1512,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Operação</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Receita no ano 1</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="15" t="n">
         <v>1000</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -846,27 +1534,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Crescimento da receita por ano</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="16" t="n">
         <v>0.1</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Aplicado nos anos 2 e 3</t>
+          <t>Aplicado do ano 2 ao ano 5</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Custos (% da receita)</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="16" t="n">
         <v>0.6</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -876,12 +1564,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Despesas (% da receita)</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.2</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -891,12 +1579,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Depreciação por ano</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="15" t="n">
         <v>50</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -906,27 +1594,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Investimento por ano (capex)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="15" t="n">
         <v>60</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Compra de máquinas e equipamentos</t>
+          <t>Compra de máquinas e equipamentos. Não passa pela DRE</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Alíquota de IR</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="16" t="n">
         <v>0.3</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -936,19 +1624,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Capital de giro</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Prazo de recebimento dos clientes (dias)</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="15" t="n">
         <v>30</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -958,12 +1646,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Prazo de pagamento aos fornecedores (dias)</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="15" t="n">
         <v>30</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -973,41 +1661,41 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Saldos iniciais (Balanço do ano 0)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Caixa</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="15" t="n">
         <v>100</v>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Imobilizado</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="15" t="n">
         <v>500</v>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Patrimônio líquido</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="15" t="n">
         <v>600</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1028,7 +1716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F14"/>
+  <dimension ref="B2:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1037,6 +1725,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1054,200 +1744,278 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="14" t="inlineStr"/>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Ano 0</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Ano 1</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Ano 2</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Ano 3</t>
         </is>
       </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Receita líquida</t>
         </is>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="19">
         <f>Premissas!$C$7</f>
         <v/>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="19">
         <f>D6*(1+Premissas!$C$8)</f>
         <v/>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="19">
         <f>E6*(1+Premissas!$C$8)</f>
         <v/>
       </c>
+      <c r="G6" s="19">
+        <f>F6*(1+Premissas!$C$8)</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>G6*(1+Premissas!$C$8)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>(−) Custos</t>
         </is>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="19">
         <f>-D6*Premissas!$C$9</f>
         <v/>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="19">
         <f>-E6*Premissas!$C$9</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="19">
         <f>-F6*Premissas!$C$9</f>
         <v/>
       </c>
+      <c r="G7" s="19">
+        <f>-G6*Premissas!$C$9</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>-H6*Premissas!$C$9</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Lucro bruto</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="20">
+      <c r="D8" s="21">
         <f>D6+D7</f>
         <v/>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="21">
         <f>E6+E7</f>
         <v/>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="21">
         <f>F6+F7</f>
         <v/>
       </c>
+      <c r="G8" s="21">
+        <f>G6+G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>H6+H7</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>(−) Despesas</t>
         </is>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="19">
         <f>-D6*Premissas!$C$10</f>
         <v/>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="19">
         <f>-E6*Premissas!$C$10</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="19">
         <f>-F6*Premissas!$C$10</f>
         <v/>
       </c>
+      <c r="G9" s="19">
+        <f>-G6*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="H9" s="19">
+        <f>-H6*Premissas!$C$10</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="20">
+      <c r="D10" s="21">
         <f>D8+D9</f>
         <v/>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <f>E8+E9</f>
         <v/>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="21">
         <f>F8+F9</f>
         <v/>
       </c>
+      <c r="G10" s="21">
+        <f>G8+G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>H8+H9</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>(−) Depreciação</t>
         </is>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="19">
         <f>-Premissas!$C$11</f>
         <v/>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="19">
         <f>-Premissas!$C$11</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="19">
         <f>-Premissas!$C$11</f>
         <v/>
       </c>
+      <c r="G11" s="19">
+        <f>-Premissas!$C$11</f>
+        <v/>
+      </c>
+      <c r="H11" s="19">
+        <f>-Premissas!$C$11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>EBIT (lucro operacional)</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="20">
+      <c r="D12" s="21">
         <f>D10+D11</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <f>E10+E11</f>
         <v/>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="21">
         <f>F10+F11</f>
         <v/>
       </c>
+      <c r="G12" s="21">
+        <f>G10+G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>H10+H11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>(−) IR</t>
         </is>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="19">
         <f>-MAX(0,D12)*Premissas!$C$13</f>
         <v/>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="19">
         <f>-MAX(0,E12)*Premissas!$C$13</f>
         <v/>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="19">
         <f>-MAX(0,F12)*Premissas!$C$13</f>
         <v/>
       </c>
+      <c r="G13" s="19">
+        <f>-MAX(0,G12)*Premissas!$C$13</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>-MAX(0,H12)*Premissas!$C$13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Lucro líquido</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="20">
+      <c r="D14" s="21">
         <f>D12+D13</f>
         <v/>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="21">
         <f>E12+E13</f>
         <v/>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="21">
         <f>F12+F13</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>G12+G13</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>H12+H13</f>
         <v/>
       </c>
     </row>
@@ -1263,7 +2031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F16"/>
+  <dimension ref="B2:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1272,6 +2040,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1289,215 +2059,291 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Ano 0</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Ano 1</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Ano 2</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Ano 3</t>
         </is>
       </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Caixa</t>
         </is>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="19">
         <f>Premissas!$C$20</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="19">
         <f>'Fluxo de Caixa'!D14</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="19">
         <f>'Fluxo de Caixa'!E14</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="19">
         <f>'Fluxo de Caixa'!F14</f>
         <v/>
       </c>
+      <c r="G6" s="19">
+        <f>'Fluxo de Caixa'!G14</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>'Fluxo de Caixa'!H14</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Contas a receber</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="22">
         <f>DRE!D6*Premissas!$C$16/360</f>
         <v/>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="22">
         <f>DRE!E6*Premissas!$C$16/360</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="22">
         <f>DRE!F6*Premissas!$C$16/360</f>
         <v/>
       </c>
+      <c r="G7" s="22">
+        <f>DRE!G6*Premissas!$C$16/360</f>
+        <v/>
+      </c>
+      <c r="H7" s="22">
+        <f>DRE!H6*Premissas!$C$16/360</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Imobilizado</t>
         </is>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="19">
         <f>Premissas!$C$21</f>
         <v/>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="22">
         <f>C8+Premissas!$C$12-Premissas!$C$11</f>
         <v/>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="22">
         <f>D8+Premissas!$C$12-Premissas!$C$11</f>
         <v/>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="22">
         <f>E8+Premissas!$C$12-Premissas!$C$11</f>
         <v/>
       </c>
+      <c r="G8" s="22">
+        <f>F8+Premissas!$C$12-Premissas!$C$11</f>
+        <v/>
+      </c>
+      <c r="H8" s="22">
+        <f>G8+Premissas!$C$12-Premissas!$C$11</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Ativo total</t>
         </is>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="21">
         <f>SUM(C6:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="21">
         <f>SUM(D6:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="21">
         <f>SUM(E6:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="21">
         <f>SUM(F6:F8)</f>
         <v/>
       </c>
+      <c r="G9" s="21">
+        <f>SUM(G6:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="21">
+        <f>SUM(H6:H8)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Passivo e patrimônio líquido</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Ano 0</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Ano 1</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Ano 2</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>Ano 3</t>
         </is>
       </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Fornecedores</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="22">
         <f>-DRE!D7*Premissas!$C$17/360</f>
         <v/>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="22">
         <f>-DRE!E7*Premissas!$C$17/360</f>
         <v/>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="22">
         <f>-DRE!F7*Premissas!$C$17/360</f>
         <v/>
       </c>
+      <c r="G12" s="22">
+        <f>-DRE!G7*Premissas!$C$17/360</f>
+        <v/>
+      </c>
+      <c r="H12" s="22">
+        <f>-DRE!H7*Premissas!$C$17/360</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Patrimônio líquido</t>
         </is>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="19">
         <f>Premissas!$C$22</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="19">
         <f>C13+DRE!D14</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="19">
         <f>D13+DRE!E14</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="19">
         <f>E13+DRE!F14</f>
         <v/>
       </c>
+      <c r="G13" s="19">
+        <f>F13+DRE!G14</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>G13+DRE!H14</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Passivo + PL</t>
         </is>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="21">
         <f>C12+C13</f>
         <v/>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="21">
         <f>D12+D13</f>
         <v/>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="21">
         <f>E12+E13</f>
         <v/>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="21">
         <f>F12+F13</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>G12+G13</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>H12+H13</f>
         <v/>
       </c>
     </row>
@@ -1507,21 +2353,36 @@
           <t>Checagem: Ativo − (Passivo + PL)</t>
         </is>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="23">
         <f>ROUND(C9-C14,6)</f>
         <v/>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="23">
         <f>ROUND(D9-D14,6)</f>
         <v/>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="23">
         <f>ROUND(E9-E14,6)</f>
         <v/>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="23">
         <f>ROUND(F9-F14,6)</f>
         <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>ROUND(G9-G14,6)</f>
+        <v/>
+      </c>
+      <c r="H16" s="23">
+        <f>ROUND(H9-H14,6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Contas a receber e fornecedores começam em zero no ano 0 (empresa-exemplo começando a operar).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1536,7 +2397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F14"/>
+  <dimension ref="B2:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1545,6 +2406,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1562,195 +2425,273 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="14" t="inlineStr"/>
-      <c r="C5" s="22" t="n"/>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="B5" s="17" t="n"/>
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Ano 1</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Ano 2</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Ano 3</t>
         </is>
       </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Lucro líquido</t>
         </is>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="19">
         <f>DRE!D14</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="19">
         <f>DRE!E14</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="19">
         <f>DRE!F14</f>
         <v/>
       </c>
+      <c r="G6" s="19">
+        <f>DRE!G14</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>DRE!H14</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>(+) Depreciação</t>
         </is>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="19">
         <f>-DRE!D11</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="19">
         <f>-DRE!E11</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="19">
         <f>-DRE!F11</f>
         <v/>
       </c>
+      <c r="G7" s="19">
+        <f>-DRE!G11</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>-DRE!H11</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>(−) Aumento de contas a receber</t>
         </is>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="22">
         <f>-(Balanço!D7-Balanço!C7)</f>
         <v/>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="22">
         <f>-(Balanço!E7-Balanço!D7)</f>
         <v/>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="22">
         <f>-(Balanço!F7-Balanço!E7)</f>
         <v/>
       </c>
+      <c r="G8" s="22">
+        <f>-(Balanço!G7-Balanço!F7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="22">
+        <f>-(Balanço!H7-Balanço!G7)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>(+) Aumento de fornecedores</t>
         </is>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="22">
         <f>Balanço!D12-Balanço!C12</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="22">
         <f>Balanço!E12-Balanço!D12</f>
         <v/>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="22">
         <f>Balanço!F12-Balanço!E12</f>
         <v/>
       </c>
+      <c r="G9" s="22">
+        <f>Balanço!G12-Balanço!F12</f>
+        <v/>
+      </c>
+      <c r="H9" s="22">
+        <f>Balanço!H12-Balanço!G12</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Caixa das operações</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="20">
+      <c r="D10" s="21">
         <f>SUM(D6:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <f>SUM(E6:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="21">
         <f>SUM(F6:F9)</f>
         <v/>
       </c>
+      <c r="G10" s="21">
+        <f>SUM(G6:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>SUM(H6:H9)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>(−) Investimentos (capex)</t>
         </is>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="19">
         <f>-Premissas!$C$12</f>
         <v/>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="19">
         <f>-Premissas!$C$12</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="19">
         <f>-Premissas!$C$12</f>
         <v/>
       </c>
+      <c r="G11" s="19">
+        <f>-Premissas!$C$12</f>
+        <v/>
+      </c>
+      <c r="H11" s="19">
+        <f>-Premissas!$C$12</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Variação do caixa</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="20">
+      <c r="D12" s="21">
         <f>D10+D11</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <f>E10+E11</f>
         <v/>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="21">
         <f>F10+F11</f>
         <v/>
       </c>
+      <c r="G12" s="21">
+        <f>G10+G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>H10+H11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Caixa inicial</t>
         </is>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="19">
         <f>Balanço!C6</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="19">
         <f>Balanço!D6</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="19">
         <f>Balanço!E6</f>
         <v/>
       </c>
+      <c r="G13" s="19">
+        <f>Balanço!F6</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>Balanço!G6</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Caixa final</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="20">
+      <c r="D14" s="21">
         <f>D13+D12</f>
         <v/>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="21">
         <f>E13+E12</f>
         <v/>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="21">
         <f>F13+F12</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>G13+G12</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>H13+H12</f>
         <v/>
       </c>
     </row>
@@ -1762,19 +2703,484 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Mapa das ligações</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>As 8 conexões que fazem os três demonstrativos virarem um modelo só. Cada uma é conferida ao vivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ano para conferir</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Digite de 1 a 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Ligação</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Sai de</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>Chega em</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Na origem</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>No destino</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>Diferença</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J7" s="25" t="inlineStr">
+        <is>
+          <t>Por que importa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>O lucro abre o Fluxo de Caixa</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>DRE · Lucro líquido</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · Lucro líquido</t>
+        </is>
+      </c>
+      <c r="F8" s="29">
+        <f>INDEX(DRE!$D$14:$H$14,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G8" s="29">
+        <f>INDEX('Fluxo de Caixa'!$D$6:$H$6,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H8" s="30">
+        <f>ROUND(F8-G8,6)</f>
+        <v/>
+      </c>
+      <c r="I8" s="31">
+        <f>IF(ABS(H8)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J8" s="28" t="inlineStr">
+        <is>
+          <t>O Fluxo de Caixa indireto começa no lucro e explica, linha a linha, por que o caixa é diferente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>O lucro soma no patrimônio líquido</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>DRE · Lucro líquido</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · aumento do PL</t>
+        </is>
+      </c>
+      <c r="F9" s="29">
+        <f>INDEX(DRE!$D$14:$H$14,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G9" s="29">
+        <f>INDEX(Balanço!$D$13:$H$13,$D$5)-INDEX(Balanço!$C$13:$G$13,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H9" s="30">
+        <f>ROUND(F9-G9,6)</f>
+        <v/>
+      </c>
+      <c r="I9" s="31">
+        <f>IF(ABS(H9)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J9" s="28" t="inlineStr">
+        <is>
+          <t>Sem ela, o Balanço fica com uma diferença exatamente igual ao lucro do ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>A depreciação volta somando no caixa</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>DRE · Depreciação</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · (+) Depreciação</t>
+        </is>
+      </c>
+      <c r="F10" s="29">
+        <f>-INDEX(DRE!$D$11:$H$11,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G10" s="29">
+        <f>INDEX('Fluxo de Caixa'!$D$7:$H$7,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H10" s="30">
+        <f>ROUND(F10-G10,6)</f>
+        <v/>
+      </c>
+      <c r="I10" s="31">
+        <f>IF(ABS(H10)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J10" s="28" t="inlineStr">
+        <is>
+          <t>Ela reduz o lucro, mas não sai do banco. Por isso é somada de volta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>A depreciação reduz o imobilizado</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>DRE · Depreciação</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · Imobilizado</t>
+        </is>
+      </c>
+      <c r="F11" s="29">
+        <f>-INDEX(DRE!$D$11:$H$11,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G11" s="29">
+        <f>INDEX(Balanço!$C$8:$G$8,$D$5)-INDEX('Fluxo de Caixa'!$D$11:$H$11,$D$5)-INDEX(Balanço!$D$8:$H$8,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H11" s="30">
+        <f>ROUND(F11-G11,6)</f>
+        <v/>
+      </c>
+      <c r="I11" s="31">
+        <f>IF(ABS(H11)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J11" s="28" t="inlineStr">
+        <is>
+          <t>O desgaste do ano sai do valor das máquinas no Balanço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="B12" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>O investimento aumenta o imobilizado</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · (−) Investimentos</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · Imobilizado</t>
+        </is>
+      </c>
+      <c r="F12" s="29">
+        <f>-INDEX('Fluxo de Caixa'!$D$11:$H$11,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G12" s="29">
+        <f>INDEX(Balanço!$D$8:$H$8,$D$5)-INDEX(Balanço!$C$8:$G$8,$D$5)-INDEX(DRE!$D$11:$H$11,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H12" s="30">
+        <f>ROUND(F12-G12,6)</f>
+        <v/>
+      </c>
+      <c r="I12" s="31">
+        <f>IF(ABS(H12)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J12" s="28" t="inlineStr">
+        <is>
+          <t>Comprar máquina tira caixa, mas não passa pela DRE: vira ativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Contas a receber consome caixa</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · Contas a receber</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · (−) Contas a receber</t>
+        </is>
+      </c>
+      <c r="F13" s="29">
+        <f>-(INDEX(Balanço!$D$7:$H$7,$D$5)-INDEX(Balanço!$C$7:$G$7,$D$5))</f>
+        <v/>
+      </c>
+      <c r="G13" s="29">
+        <f>INDEX('Fluxo de Caixa'!$D$8:$H$8,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H13" s="30">
+        <f>ROUND(F13-G13,6)</f>
+        <v/>
+      </c>
+      <c r="I13" s="31">
+        <f>IF(ABS(H13)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J13" s="28" t="inlineStr">
+        <is>
+          <t>Venda a prazo entra no lucro, mas o dinheiro ainda está com o cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Fornecedores seguram caixa</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · Fornecedores</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · (+) Fornecedores</t>
+        </is>
+      </c>
+      <c r="F14" s="29">
+        <f>INDEX(Balanço!$D$12:$H$12,$D$5)-INDEX(Balanço!$C$12:$G$12,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>INDEX('Fluxo de Caixa'!$D$9:$H$9,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H14" s="30">
+        <f>ROUND(F14-G14,6)</f>
+        <v/>
+      </c>
+      <c r="I14" s="31">
+        <f>IF(ABS(H14)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J14" s="28" t="inlineStr">
+        <is>
+          <t>Comprar a prazo entra no custo, mas o dinheiro só sai depois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>O caixa final fecha o Balanço</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa · Caixa final</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>Balanço · Caixa</t>
+        </is>
+      </c>
+      <c r="F15" s="29">
+        <f>INDEX('Fluxo de Caixa'!$D$14:$H$14,$D$5)</f>
+        <v/>
+      </c>
+      <c r="G15" s="29">
+        <f>INDEX(Balanço!$D$6:$H$6,$D$5)</f>
+        <v/>
+      </c>
+      <c r="H15" s="30">
+        <f>ROUND(F15-G15,6)</f>
+        <v/>
+      </c>
+      <c r="I15" s="31">
+        <f>IF(ABS(H15)&lt;0.01,"Ligada","Quebrada")</f>
+        <v/>
+      </c>
+      <c r="J15" s="28" t="inlineStr">
+        <is>
+          <t>É a última ligação: com ela, Ativo = Passivo + PL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Ligações funcionando</t>
+        </is>
+      </c>
+      <c r="D17" s="3">
+        <f>COUNTIF(I8:I15,"Ligada")&amp;" de 8"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Para ver uma ligação quebrar, faça o exercício 5 da aba Exercícios.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I8:I15">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>I8="Ligada"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>I8="Quebrada"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="D5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Ano inválido" error="Digite um ano de 1 a 5." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0015803D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F10"/>
+  <dimension ref="B2:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1792,122 +3198,881 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="14" t="inlineStr"/>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Ano 0</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Ano 1</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Ano 2</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Ano 3</t>
         </is>
       </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Ativo − (Passivo + PL)</t>
         </is>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="19">
         <f>Balanço!C16</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="19">
         <f>Balanço!D16</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="19">
         <f>Balanço!E16</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="19">
         <f>Balanço!F16</f>
         <v/>
       </c>
+      <c r="G6" s="19">
+        <f>Balanço!G16</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>Balanço!H16</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Caixa do Fluxo de Caixa − Caixa do Balanço</t>
         </is>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="22">
         <f>ROUND('Fluxo de Caixa'!D14-Balanço!D6,6)</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="22">
         <f>ROUND('Fluxo de Caixa'!E14-Balanço!E6,6)</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="22">
         <f>ROUND('Fluxo de Caixa'!F14-Balanço!F6,6)</f>
         <v/>
       </c>
+      <c r="G7" s="22">
+        <f>ROUND('Fluxo de Caixa'!G14-Balanço!G6,6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="22">
+        <f>ROUND('Fluxo de Caixa'!H14-Balanço!H6,6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Lucro da DRE − aumento do PL</t>
+        </is>
+      </c>
+      <c r="D8" s="22">
+        <f>ROUND(DRE!D14-(Balanço!D13-Balanço!C13),6)</f>
+        <v/>
+      </c>
+      <c r="E8" s="22">
+        <f>ROUND(DRE!E14-(Balanço!E13-Balanço!D13),6)</f>
+        <v/>
+      </c>
+      <c r="F8" s="22">
+        <f>ROUND(DRE!F14-(Balanço!F13-Balanço!E13),6)</f>
+        <v/>
+      </c>
+      <c r="G8" s="22">
+        <f>ROUND(DRE!G14-(Balanço!G13-Balanço!F13),6)</f>
+        <v/>
+      </c>
+      <c r="H8" s="22">
+        <f>ROUND(DRE!H14-(Balanço!H13-Balanço!G13),6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Situação</t>
         </is>
       </c>
-      <c r="C8" s="23">
-        <f>IF(AND(ABS(C6)&lt;0.01,ABS(N(C7))&lt;0.01),"Fecha","Não fecha")</f>
-        <v/>
-      </c>
-      <c r="D8" s="23">
-        <f>IF(AND(ABS(D6)&lt;0.01,ABS(N(D7))&lt;0.01),"Fecha","Não fecha")</f>
-        <v/>
-      </c>
-      <c r="E8" s="23">
-        <f>IF(AND(ABS(E6)&lt;0.01,ABS(N(E7))&lt;0.01),"Fecha","Não fecha")</f>
-        <v/>
-      </c>
-      <c r="F8" s="23">
-        <f>IF(AND(ABS(F6)&lt;0.01,ABS(N(F7))&lt;0.01),"Fecha","Não fecha")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="C9" s="32">
+        <f>IF(AND(ABS(C6)&lt;0.01,ABS(N(C7))&lt;0.01,ABS(N(C8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+      <c r="D9" s="32">
+        <f>IF(AND(ABS(D6)&lt;0.01,ABS(N(D7))&lt;0.01,ABS(N(D8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+      <c r="E9" s="32">
+        <f>IF(AND(ABS(E6)&lt;0.01,ABS(N(E7))&lt;0.01,ABS(N(E8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+      <c r="F9" s="32">
+        <f>IF(AND(ABS(F6)&lt;0.01,ABS(N(F7))&lt;0.01,ABS(N(F8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
+        <f>IF(AND(ABS(G6)&lt;0.01,ABS(N(G7))&lt;0.01,ABS(N(G8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+      <c r="H9" s="32">
+        <f>IF(AND(ABS(H6)&lt;0.01,ABS(N(H7))&lt;0.01,ABS(N(H8))&lt;0.01),"Fecha","Não fecha")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Resultado do modelo</t>
         </is>
       </c>
-      <c r="C10" s="24">
-        <f>IF(COUNTIF(C8:F8,"Fecha")=4,"✓ O modelo fecha nos 3 anos","✗ Há uma ligação quebrada")</f>
+      <c r="C11" s="33">
+        <f>IF(COUNTIF(C9:H9,"Fecha")=6,"✓ O modelo fecha nos 5 anos","✗ Há uma ligação quebrada")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:H11"/>
   </mergeCells>
-  <conditionalFormatting sqref="C8:F8">
+  <conditionalFormatting sqref="C9:H9">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEFT(C8,1)="F"</formula>
+      <formula>LEFT(C9,1)="F"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT(C8,1)="N"</formula>
+      <formula>LEFT(C9,1)="N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C10:F10">
+  <conditionalFormatting sqref="C11:H11">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>LEFT($C$10,1)="✓"</formula>
+      <formula>LEFT($C$11,1)="✓"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="1">
-      <formula>LEFT($C$10,1)="✗"</formula>
+      <formula>LEFT($C$11,1)="✗"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00070D24"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Lucro x Caixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>R$ mil. Por que o caixa das operações não é igual ao lucro, ano a ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="17" t="n"/>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 1</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 2</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 3</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Lucro líquido</t>
+        </is>
+      </c>
+      <c r="D6" s="19">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="E6" s="19">
+        <f>DRE!E14</f>
+        <v/>
+      </c>
+      <c r="F6" s="19">
+        <f>DRE!F14</f>
+        <v/>
+      </c>
+      <c r="G6" s="19">
+        <f>DRE!G14</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>DRE!H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>(+) Depreciação</t>
+        </is>
+      </c>
+      <c r="D7" s="19">
+        <f>'Fluxo de Caixa'!D7</f>
+        <v/>
+      </c>
+      <c r="E7" s="19">
+        <f>'Fluxo de Caixa'!E7</f>
+        <v/>
+      </c>
+      <c r="F7" s="19">
+        <f>'Fluxo de Caixa'!F7</f>
+        <v/>
+      </c>
+      <c r="G7" s="19">
+        <f>'Fluxo de Caixa'!G7</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>'Fluxo de Caixa'!H7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>(−) Aumento de contas a receber</t>
+        </is>
+      </c>
+      <c r="D8" s="19">
+        <f>'Fluxo de Caixa'!D8</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>'Fluxo de Caixa'!E8</f>
+        <v/>
+      </c>
+      <c r="F8" s="19">
+        <f>'Fluxo de Caixa'!F8</f>
+        <v/>
+      </c>
+      <c r="G8" s="19">
+        <f>'Fluxo de Caixa'!G8</f>
+        <v/>
+      </c>
+      <c r="H8" s="19">
+        <f>'Fluxo de Caixa'!H8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>(+) Aumento de fornecedores</t>
+        </is>
+      </c>
+      <c r="D9" s="19">
+        <f>'Fluxo de Caixa'!D9</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>'Fluxo de Caixa'!E9</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>'Fluxo de Caixa'!F9</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>'Fluxo de Caixa'!G9</f>
+        <v/>
+      </c>
+      <c r="H9" s="19">
+        <f>'Fluxo de Caixa'!H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Caixa das operações</t>
+        </is>
+      </c>
+      <c r="D10" s="21">
+        <f>SUM(D6:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>SUM(E6:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>SUM(F6:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUM(G6:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>SUM(H6:H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Diferença: caixa − lucro</t>
+        </is>
+      </c>
+      <c r="D11" s="22">
+        <f>D10-D6</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>E10-E6</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>F10-F6</f>
+        <v/>
+      </c>
+      <c r="G11" s="22">
+        <f>G10-G6</f>
+        <v/>
+      </c>
+      <c r="H11" s="22">
+        <f>H10-H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Conversão do lucro em caixa</t>
+        </is>
+      </c>
+      <c r="D12" s="34">
+        <f>IF(D6=0,0,D10/D6)</f>
+        <v/>
+      </c>
+      <c r="E12" s="34">
+        <f>IF(E6=0,0,E10/E6)</f>
+        <v/>
+      </c>
+      <c r="F12" s="34">
+        <f>IF(F6=0,0,F10/F6)</f>
+        <v/>
+      </c>
+      <c r="G12" s="34">
+        <f>IF(G6=0,0,G10/G6)</f>
+        <v/>
+      </c>
+      <c r="H12" s="34">
+        <f>IF(H6=0,0,H10/H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Ano 1</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Ano 2</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Ano 3</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Margem EBITDA</t>
+        </is>
+      </c>
+      <c r="D15" s="34">
+        <f>IF(DRE!D6=0,0,DRE!D10/DRE!D6)</f>
+        <v/>
+      </c>
+      <c r="E15" s="34">
+        <f>IF(DRE!E6=0,0,DRE!E10/DRE!E6)</f>
+        <v/>
+      </c>
+      <c r="F15" s="34">
+        <f>IF(DRE!F6=0,0,DRE!F10/DRE!F6)</f>
+        <v/>
+      </c>
+      <c r="G15" s="34">
+        <f>IF(DRE!G6=0,0,DRE!G10/DRE!G6)</f>
+        <v/>
+      </c>
+      <c r="H15" s="34">
+        <f>IF(DRE!H6=0,0,DRE!H10/DRE!H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Margem líquida</t>
+        </is>
+      </c>
+      <c r="D16" s="34">
+        <f>IF(DRE!D6=0,0,DRE!D14/DRE!D6)</f>
+        <v/>
+      </c>
+      <c r="E16" s="34">
+        <f>IF(DRE!E6=0,0,DRE!E14/DRE!E6)</f>
+        <v/>
+      </c>
+      <c r="F16" s="34">
+        <f>IF(DRE!F6=0,0,DRE!F14/DRE!F6)</f>
+        <v/>
+      </c>
+      <c r="G16" s="34">
+        <f>IF(DRE!G6=0,0,DRE!G14/DRE!G6)</f>
+        <v/>
+      </c>
+      <c r="H16" s="34">
+        <f>IF(DRE!H6=0,0,DRE!H14/DRE!H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Prazo médio de recebimento</t>
+        </is>
+      </c>
+      <c r="D17" s="35">
+        <f>IF(DRE!D6=0,0,Balanço!D7/DRE!D6*360)</f>
+        <v/>
+      </c>
+      <c r="E17" s="35">
+        <f>IF(DRE!E6=0,0,Balanço!E7/DRE!E6*360)</f>
+        <v/>
+      </c>
+      <c r="F17" s="35">
+        <f>IF(DRE!F6=0,0,Balanço!F7/DRE!F6*360)</f>
+        <v/>
+      </c>
+      <c r="G17" s="35">
+        <f>IF(DRE!G6=0,0,Balanço!G7/DRE!G6*360)</f>
+        <v/>
+      </c>
+      <c r="H17" s="35">
+        <f>IF(DRE!H6=0,0,Balanço!H7/DRE!H6*360)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Prazo médio de pagamento</t>
+        </is>
+      </c>
+      <c r="D18" s="35">
+        <f>IF(DRE!D7=0,0,Balanço!D12/-DRE!D7*360)</f>
+        <v/>
+      </c>
+      <c r="E18" s="35">
+        <f>IF(DRE!E7=0,0,Balanço!E12/-DRE!E7*360)</f>
+        <v/>
+      </c>
+      <c r="F18" s="35">
+        <f>IF(DRE!F7=0,0,Balanço!F12/-DRE!F7*360)</f>
+        <v/>
+      </c>
+      <c r="G18" s="35">
+        <f>IF(DRE!G7=0,0,Balanço!G12/-DRE!G7*360)</f>
+        <v/>
+      </c>
+      <c r="H18" s="35">
+        <f>IF(DRE!H7=0,0,Balanço!H12/-DRE!H7*360)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Caixa no fim do ano</t>
+        </is>
+      </c>
+      <c r="D19" s="19">
+        <f>Balanço!D6</f>
+        <v/>
+      </c>
+      <c r="E19" s="19">
+        <f>Balanço!E6</f>
+        <v/>
+      </c>
+      <c r="F19" s="19">
+        <f>Balanço!F6</f>
+        <v/>
+      </c>
+      <c r="G19" s="19">
+        <f>Balanço!G6</f>
+        <v/>
+      </c>
+      <c r="H19" s="19">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Conversão acima de 100%: a operação gera mais caixa do que lucro. Abaixo: o lucro está preso no capital de giro.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F59E0B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Exercícios: teste as ligações</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Faça um de cada vez e volte o valor original antes do próximo. Os números à direita mudam na hora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>Experimento</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>O que fazer</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="inlineStr">
+        <is>
+          <t>O que observar</t>
+        </is>
+      </c>
+      <c r="F5" s="37" t="inlineStr">
+        <is>
+          <t>Lucro ano 1</t>
+        </is>
+      </c>
+      <c r="G5" s="37" t="inlineStr">
+        <is>
+          <t>Caixa operações ano 1</t>
+        </is>
+      </c>
+      <c r="H5" s="37" t="inlineStr">
+        <is>
+          <t>Caixa final ano 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="B6" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>Lucro não é caixa</t>
+        </is>
+      </c>
+      <c r="D6" s="40" t="inlineStr">
+        <is>
+          <t>Na aba Premissas, mude o prazo de recebimento de 30 para 120 dias.</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>O lucro não muda. O caixa das operações cai: um terço das vendas do ano fica com o cliente.</t>
+        </is>
+      </c>
+      <c r="F6" s="42">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="G6" s="42">
+        <f>'Fluxo de Caixa'!D10</f>
+        <v/>
+      </c>
+      <c r="H6" s="42">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="B7" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
+        <is>
+          <t>O fornecedor também financia</t>
+        </is>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>Mude o prazo de pagamento aos fornecedores de 30 para 60 dias.</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>O caixa sobe sem o lucro mudar: você vende antes de pagar.</t>
+        </is>
+      </c>
+      <c r="F7" s="42">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="G7" s="42">
+        <f>'Fluxo de Caixa'!D10</f>
+        <v/>
+      </c>
+      <c r="H7" s="42">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="B8" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="39" t="inlineStr">
+        <is>
+          <t>Depreciação e imposto</t>
+        </is>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>Mude a depreciação de 50 para 0.</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>O lucro sobe, mas o caixa cai. Sem a depreciação, o lucro tributável aumenta e você paga mais IR.</t>
+        </is>
+      </c>
+      <c r="F8" s="42">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="G8" s="42">
+        <f>'Fluxo de Caixa'!D10</f>
+        <v/>
+      </c>
+      <c r="H8" s="42">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="B9" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>Investimento não passa pela DRE</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>Mude o investimento por ano (capex) de 60 para 200.</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>O lucro fica igual. O caixa final cai 140 por ano e o imobilizado cresce no Balanço.</t>
+        </is>
+      </c>
+      <c r="F9" s="42">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="G9" s="42">
+        <f>'Fluxo de Caixa'!D10</f>
+        <v/>
+      </c>
+      <c r="H9" s="42">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="B10" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>Quebre uma ligação</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>Na aba Balanço, célula D13, apague o trecho +DRE!D14 da fórmula. Depois desfaça com Ctrl+Z.</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>A aba Checagem mostra diferença igual ao lucro e a aba Ligações marca a ligação 2 como Quebrada.</t>
+        </is>
+      </c>
+      <c r="F10" s="42">
+        <f>DRE!D14</f>
+        <v/>
+      </c>
+      <c r="G10" s="42">
+        <f>'Fluxo de Caixa'!D10</f>
+        <v/>
+      </c>
+      <c r="H10" s="42">
+        <f>Balanço!H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Valores originais</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Prazo de clientes 30 · Prazo de fornecedores 30 · Depreciação 50 · Capex 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Resultado do modelo agora</t>
+        </is>
+      </c>
+      <c r="D13" s="4">
+        <f>Checagem!C11</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEFT($D$13,1)="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>LEFT($D$13,1)="✗"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>